<commit_message>
Record left arm v2 bring-up tuning
</commit_message>
<xml_diff>
--- a/左臂电机ID备忘.xlsx
+++ b/左臂电机ID备忘.xlsx
@@ -523,7 +523,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -816,6 +816,90 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>左腕上下</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>DM4310</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>0x19</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>0x29</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>Existing wrist up/down joint in left_arm_controller.py; located after arm_roll and before new wrist-side joint</t>
+        </is>
+      </c>
+      <c r="I8" s="7" t="inlineStr">
+        <is>
+          <t>installed/tested in controller</t>
+        </is>
+      </c>
+      <c r="J8" s="7" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>左腕左右</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>DM4310</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>0x1A</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>0x2A</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>Installed on 2026-07-18. Wrist section length increased by 8.5 cm; verify zero/sign and update geometry model after calibration.</t>
+        </is>
+      </c>
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t>installed, needs zero/sign test</t>
+        </is>
+      </c>
+      <c r="J9" s="7" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
@@ -830,7 +914,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1491,7 +1575,11 @@
           <t>右肩前摆</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr"/>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>DM4340</t>
+        </is>
+      </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
           <t>0x13</t>
@@ -1510,7 +1598,7 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>右臂</t>
+          <t>Right arm shoulder front; ID set on motor, reserved original right-arm planning ID</t>
         </is>
       </c>
     </row>
@@ -1675,6 +1763,78 @@
       <c r="H25" s="4" t="inlineStr">
         <is>
           <t>新增左爪；不在原图规划中；按顺序续编</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>左腕上下</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>DM4310</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>0x19</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>0x29</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="n">
+        <v>41</v>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>Left wrist up/down; existing controller joint name wrist</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>左腕左右</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>DM4310</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>0x1A</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>0x2A</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="n">
+        <v>42</v>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>Installed on 2026-07-18. Wrist section length increased by 8.5 cm; verify zero/sign and update geometry model after calibration.</t>
         </is>
       </c>
     </row>
@@ -1692,7 +1852,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1858,6 +2018,174 @@
       <c r="G4" s="7" t="n"/>
       <c r="H4" s="7" t="n"/>
     </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>ID planning</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>左腕左右</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>0x1A</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>0x2A</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>Reserve final ID for new left wrist-side joint</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>recorded, pending install/test</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>Changed from temporary 0x13/0x23 to 0x1A/0x2A so right shoulder front keeps original 0x13/0x23</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>USB-CAN / ID setup</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>右肩前摆</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>0x13</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>0x23</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>Right shoulder front motor ID configured</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>recorded</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>Motor model recorded as DM4340; verify read/status and small motion before powered assembly</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>ID record</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>左腕上下</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>0x19</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>0x29</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>Backfill existing wrist up/down ID from controller code</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>recorded</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>left_arm_controller.py joint name: wrist; DM4310</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Mechanical install</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>左腕左右</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>0x1A</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>0x2A</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>Left wrist-side joint installed; wrist section +8.5 cm</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>installed, needs zero/sign test</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>Do not fold the +8.5 cm into IK until the new joint zero, sign, and effective link segment are verified.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>